<commit_message>
Keep only ebid-lcs-automation, removed other projects
</commit_message>
<xml_diff>
--- a/OpenCartFramework/testData/Global_TestData.xlsx
+++ b/OpenCartFramework/testData/Global_TestData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="13"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="14"/>
   </bookViews>
   <sheets>
     <sheet name="AddFollowUP1" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,6 +22,7 @@
     <sheet name="SiteVisit" sheetId="12" state="visible" r:id="rId14"/>
     <sheet name="Remedial" sheetId="13" state="visible" r:id="rId15"/>
     <sheet name="LegalOrder" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="Calendar" sheetId="15" state="visible" r:id="rId17"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="477">
   <si>
     <t xml:space="preserve">Comm type</t>
   </si>
@@ -1398,15 +1399,82 @@
   </si>
   <si>
     <t xml:space="preserve">Legal order final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIELD_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INPUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXPECTED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECK_TYPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAL_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">checkbox</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PTP checkbox should be selected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAL_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site Visited checkbox should be selected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAL_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Next Court Case checkbox should be selected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAL_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Next Hearing checkbox should be selected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAL_05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Call checkbox should be selected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAL_06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mail checkbox should be selected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAL_07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SITE VISIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site Visit checkbox should be selected</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -1521,7 +1589,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1624,6 +1692,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -3261,6 +3333,189 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="31.57"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>455</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>456</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>457</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>458</v>
+      </c>
+      <c r="F1" s="22" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="23" t="s">
+        <v>460</v>
+      </c>
+      <c r="B2" s="23" t="n">
+        <v>99</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>461</v>
+      </c>
+      <c r="D2" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>462</v>
+      </c>
+      <c r="F2" s="23" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="23" t="s">
+        <v>463</v>
+      </c>
+      <c r="B3" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>461</v>
+      </c>
+      <c r="D3" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>464</v>
+      </c>
+      <c r="F3" s="23" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="23" t="s">
+        <v>465</v>
+      </c>
+      <c r="B4" s="23" t="n">
+        <v>101</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>461</v>
+      </c>
+      <c r="D4" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>466</v>
+      </c>
+      <c r="F4" s="23" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="s">
+        <v>467</v>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>102</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>461</v>
+      </c>
+      <c r="D5" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>468</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="23" t="s">
+        <v>469</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>461</v>
+      </c>
+      <c r="D6" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>470</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
+        <v>471</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>472</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>461</v>
+      </c>
+      <c r="D7" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>473</v>
+      </c>
+      <c r="F7" s="23" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="23" t="s">
+        <v>474</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>475</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>461</v>
+      </c>
+      <c r="D8" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>476</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>186</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>